<commit_message>
implement tournament management page with bracket generation, mat assignment, and registration tracking components
</commit_message>
<xml_diff>
--- a/public/templates/players_import_template.xlsx
+++ b/public/templates/players_import_template.xlsx
@@ -399,10 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
-  <cols>
-    <col min="1" max="1" width="110.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:A20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -491,43 +488,29 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>11. Delete the two sample rows before importing your real data.</v>
+        <v>11. Payment Status (optional) marks whether the player has paid for this tournament. Use PAID / YES / TRUE / Y / 1 for paid — anything else (including blank) is treated as unpaid.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>12. Save as .xlsx, .xls, or .csv before uploading. Max file size: 5 MB.</v>
+        <v>12. Delete the two sample rows before importing your real data.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>13. Save as .xlsx, .xls, or .csv before uploading. Max file size: 5 MB.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="17.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:R3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -581,6 +564,9 @@
       <c r="Q1" t="str">
         <v>Coach ID</v>
       </c>
+      <c r="R1" t="str">
+        <v>Payment Status</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -634,6 +620,9 @@
       <c r="Q2" t="str">
         <v>9876500001</v>
       </c>
+      <c r="R2" t="str">
+        <v>PAID</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -687,10 +676,13 @@
       <c r="Q3" t="str">
         <v/>
       </c>
+      <c r="R3" t="str">
+        <v>UNPAID</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -698,10 +690,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B293"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>